<commit_message>
/Production : removed production files to update
</commit_message>
<xml_diff>
--- a/Hardware/production/Flight Controller.csv.xlsx
+++ b/Hardware/production/Flight Controller.csv.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saleh\Desktop\Saleh Uni\sem 7\senior year project\Flight Controller\Hardware\production\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Work and Study\Desktop\SAL-FC\Hardware\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8FF64B-F582-4F2E-B400-404A08295332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8099E558-6709-413C-BDA1-1BD98D17FB02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{EE1FF5F6-602B-4445-90C3-6F00E465E91C}"/>
   </bookViews>
@@ -284,9 +284,6 @@
   </si>
   <si>
     <t>5.1k</t>
-  </si>
-  <si>
-    <t>Resistor_SMD:R_0402_1005Metric</t>
   </si>
   <si>
     <t>R3,R5</t>
@@ -534,12 +531,15 @@
       <t>@100Mhz</t>
     </r>
   </si>
+  <si>
+    <t>Resistor_SMD:R_0402</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1403,18 +1403,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37BC14FF-DD66-40C3-902A-DA2A77DEECF1}">
   <dimension ref="A1:E66"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="76.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1796875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="60.1796875" customWidth="1"/>
-    <col min="5" max="5" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.1640625" customWidth="1"/>
+    <col min="5" max="5" width="9.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1429,7 +1429,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1527,7 +1527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1597,7 +1597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -1706,13 +1706,13 @@
         <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D21" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>52</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -1796,7 +1796,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>65</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
         <v>70</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
         <v>79</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>86</v>
       </c>
@@ -1922,26 +1922,26 @@
         <v>87</v>
       </c>
       <c r="D36" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>89</v>
       </c>
       <c r="B37" s="1">
         <v>2</v>
       </c>
       <c r="C37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
         <v>90</v>
-      </c>
-      <c r="D37" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>91</v>
       </c>
       <c r="B38" s="1">
         <v>1</v>
@@ -1950,68 +1950,68 @@
         <v>49.9</v>
       </c>
       <c r="D38" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
+        <v>91</v>
+      </c>
+      <c r="B39" s="1">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B39" s="1">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
         <v>93</v>
       </c>
-      <c r="D39" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="B40" s="1">
+        <v>1</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="1">
-        <v>1</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
         <v>95</v>
       </c>
-      <c r="D40" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="B41" s="1">
+        <v>1</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B41" s="1">
-        <v>1</v>
-      </c>
-      <c r="C41" s="1" t="s">
+      <c r="D41" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
         <v>97</v>
       </c>
-      <c r="D41" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="B42" s="1">
+        <v>1</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B42" s="1">
-        <v>1</v>
-      </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
         <v>99</v>
-      </c>
-      <c r="D42" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>100</v>
       </c>
       <c r="B43" s="1">
         <v>3</v>
@@ -2020,29 +2020,29 @@
         <v>0</v>
       </c>
       <c r="D43" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
       <c r="A44" t="s">
+        <v>100</v>
+      </c>
+      <c r="B44" s="1">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B44" s="1">
-        <v>1</v>
-      </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" t="s">
         <v>102</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>103</v>
       </c>
-      <c r="E44" t="s">
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>105</v>
       </c>
       <c r="B45" s="1">
         <v>4</v>
@@ -2051,40 +2051,40 @@
         <v>330</v>
       </c>
       <c r="D45" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B46" s="1">
         <v>5</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
         <v>107</v>
-      </c>
-      <c r="D46" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>108</v>
       </c>
       <c r="B47" s="1">
         <v>4</v>
       </c>
       <c r="C47" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D47" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
         <v>109</v>
-      </c>
-      <c r="D47" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>110</v>
       </c>
       <c r="B48" s="1">
         <v>2</v>
@@ -2093,12 +2093,12 @@
         <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B49" s="1">
         <v>1</v>
@@ -2107,255 +2107,261 @@
         <v>120</v>
       </c>
       <c r="D49" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B50" s="1">
         <v>2</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D50" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
         <v>113</v>
       </c>
-      <c r="D50" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+      <c r="B51" s="1">
+        <v>1</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B51" s="1">
-        <v>1</v>
-      </c>
-      <c r="C51" s="1" t="s">
+      <c r="D51" t="s">
         <v>115</v>
       </c>
-      <c r="D51" t="s">
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+      <c r="B52" s="1">
+        <v>1</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B52" s="1">
-        <v>1</v>
-      </c>
-      <c r="C52" s="1" t="s">
+      <c r="D52" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
         <v>118</v>
       </c>
-      <c r="D52" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+      <c r="B53" s="1">
+        <v>1</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B53" s="1">
-        <v>1</v>
-      </c>
-      <c r="C53" s="1" t="s">
+      <c r="D53" t="s">
         <v>120</v>
       </c>
-      <c r="D53" t="s">
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+      <c r="B54" s="1">
+        <v>1</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B54" s="1">
-        <v>1</v>
-      </c>
-      <c r="C54" s="1" t="s">
+      <c r="D54" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
         <v>123</v>
       </c>
-      <c r="D54" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+      <c r="B55" s="1">
+        <v>1</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="1">
-        <v>1</v>
-      </c>
-      <c r="C55" s="1" t="s">
+      <c r="D55" t="s">
         <v>125</v>
       </c>
-      <c r="D55" t="s">
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+      <c r="B56" s="1">
+        <v>1</v>
+      </c>
+      <c r="C56" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B56" s="1">
-        <v>1</v>
-      </c>
-      <c r="C56" s="1" t="s">
+      <c r="D56" t="s">
         <v>128</v>
       </c>
-      <c r="D56" t="s">
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+      <c r="B57" s="1">
+        <v>1</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B57" s="1">
-        <v>1</v>
-      </c>
-      <c r="C57" s="1" t="s">
+      <c r="D57" t="s">
         <v>131</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>132</v>
       </c>
-      <c r="E57" t="s">
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+      <c r="B58" s="1">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B58" s="1">
-        <v>1</v>
-      </c>
-      <c r="C58" s="1" t="s">
+      <c r="D58" t="s">
         <v>135</v>
       </c>
-      <c r="D58" t="s">
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+      <c r="B59" s="1">
+        <v>1</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B59" s="1">
-        <v>1</v>
-      </c>
-      <c r="C59" s="1" t="s">
+      <c r="D59" t="s">
         <v>138</v>
       </c>
-      <c r="D59" t="s">
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+      <c r="B60" s="1">
+        <v>1</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B60" s="1">
-        <v>1</v>
-      </c>
-      <c r="C60" s="1" t="s">
+      <c r="D60" t="s">
         <v>141</v>
       </c>
-      <c r="D60" t="s">
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+      <c r="B61" s="1">
+        <v>1</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="1">
-        <v>1</v>
-      </c>
-      <c r="C61" s="1" t="s">
+      <c r="D61" t="s">
         <v>144</v>
       </c>
-      <c r="D61" t="s">
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+      <c r="B62" s="1">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B62" s="1">
-        <v>1</v>
-      </c>
-      <c r="C62" s="1" t="s">
+      <c r="D62" t="s">
         <v>147</v>
       </c>
-      <c r="D62" t="s">
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+      <c r="B63" s="1">
+        <v>1</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="1">
-        <v>1</v>
-      </c>
-      <c r="C63" s="1" t="s">
+      <c r="D63" t="s">
         <v>150</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>151</v>
       </c>
-      <c r="E63" t="s">
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+      <c r="B64" s="1">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B64" s="1">
-        <v>1</v>
-      </c>
-      <c r="C64" s="1" t="s">
+      <c r="D64" t="s">
         <v>154</v>
       </c>
-      <c r="D64" t="s">
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+      <c r="B65" s="1">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B65" s="1">
-        <v>1</v>
-      </c>
-      <c r="C65" s="1" t="s">
+      <c r="D65" t="s">
         <v>157</v>
       </c>
-      <c r="D65" t="s">
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+      <c r="B66" s="1">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B66" s="1">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="s">
+      <c r="D66" t="s">
         <v>160</v>
-      </c>
-      <c r="D66" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9f5c8052-b1ea-40d1-8cd5-ea0c204ca84f}" enabled="1" method="Standard" siteId="{19e51c11-d919-4a98-899d-9b9dc33f4e04}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>